<commit_message>
Localization support, output suffix, run report, detailed VRAM usage report, download mirror for mainland China, one pass finalize, save last n consoles, minor bug fixes
</commit_message>
<xml_diff>
--- a/ChitraMaya-Roadmap.xlsx
+++ b/ChitraMaya-Roadmap.xlsx
@@ -7,9 +7,11 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Next Drop (proposed)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Updates" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roadmap'!$A$1:$J$91</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roadmap'!$A$1:$J$166</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -17,8 +19,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+  </numFmts>
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,6 +32,11 @@
     </font>
     <font>
       <name val="Aptos Narrow"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -51,13 +60,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -423,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J91"/>
+  <dimension ref="A1:J167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1792,7 +1802,7 @@
       <c r="I32" s="1" t="n"/>
       <c r="J32" s="1" t="n"/>
     </row>
-    <row r="33" ht="180" customHeight="1">
+    <row r="33" hidden="1" ht="180" customHeight="1">
       <c r="A33" s="1" t="inlineStr">
         <is>
           <t>CM-032</t>
@@ -2052,7 +2062,7 @@
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="C39" s="1" t="inlineStr">
@@ -2338,7 +2348,7 @@
       <c r="I45" s="1" t="n"/>
       <c r="J45" s="1" t="n"/>
     </row>
-    <row r="46" ht="60" customHeight="1">
+    <row r="46" hidden="1" ht="60" customHeight="1">
       <c r="A46" s="1" t="inlineStr">
         <is>
           <t>CM-045</t>
@@ -2380,7 +2390,7 @@
       <c r="I46" s="1" t="n"/>
       <c r="J46" s="1" t="n"/>
     </row>
-    <row r="47" ht="30" customHeight="1">
+    <row r="47" hidden="1" ht="30" customHeight="1">
       <c r="A47" s="1" t="inlineStr">
         <is>
           <t>CM-046</t>
@@ -2393,7 +2403,7 @@
       </c>
       <c r="C47" s="1" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D47" s="1" t="inlineStr">
@@ -2408,7 +2418,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>showDialog(title, msg) for all popups - custom styled, not browser-native. Ported from gSwapper RM-026.</t>
+          <t>showDialog(title, msg) for all popups - custom styled, not browser-native. Ported from gSwapper RM-026. || UPDATE 2026-09-11: Shipped: showConfirm()/modal overlay replaces confirm/alert (Batch 13 modal work; used by presets delete, Reset Defaults). v1.70.00.</t>
         </is>
       </c>
       <c r="G47" s="1" t="inlineStr">
@@ -2450,7 +2460,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Write build_info.json after each compile: hostname, GPU model, TensorRT version, compile date, per-engine compile time + scratch memory. Diagnoses cross-machine perf differences and which machine built which engines. Ties to Model Management (CM-029). Ported from gSwapper RM-031.</t>
+          <t>Write build_info.json after each compile: hostname, GPU model, TensorRT version, compile date, per-engine compile time + scratch memory. Diagnoses cross-machine perf differences and which machine built which engines. Ties to Model Management (CM-029). Ported from gSwapper RM-031. || UPDATE 2026-09-11: Superseded by CM-151 (engine manifest with build stamp + provenance).</t>
         </is>
       </c>
       <c r="G48" s="1" t="inlineStr">
@@ -3010,7 +3020,7 @@
       <c r="I61" s="1" t="n"/>
       <c r="J61" s="1" t="n"/>
     </row>
-    <row r="62" ht="90" customHeight="1">
+    <row r="62" hidden="1" ht="90" customHeight="1">
       <c r="A62" s="1" t="inlineStr">
         <is>
           <t>CM-061</t>
@@ -3023,7 +3033,7 @@
       </c>
       <c r="C62" s="1" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D62" s="1" t="inlineStr">
@@ -3038,7 +3048,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Run-time detection imgsz is hardwired to 640 on the UI path (MosaicConfig has no field; to_pipeline_config never sets it). 960-imgsz detection is CLI-only (--det-imgsz). Add a Detection Image Size dial to the Control Panel, wire it through MosaicConfig + the pipeline rebuild key, and snap/select to the selected detection engine's compiled size (as Max Clip does for restoration; a .pt is dynamic). Unblocks the 640-vs-960 comparison from the UI. From CM-049.</t>
+          <t>Run-time detection imgsz is hardwired to 640 on the UI path (MosaicConfig has no field; to_pipeline_config never sets it). 960-imgsz detection is CLI-only (--det-imgsz). Add a Detection Image Size dial to the Control Panel, wire it through MosaicConfig + the pipeline rebuild key, and snap/select to the selected detection engine's compiled size (as Max Clip does for restoration; a .pt is dynamic). Unblocks the 640-vs-960 comparison from the UI. From CM-049. || UPDATE 2026-09-11: Shipped: Detection Image Size dial (Batch 17, v1.20/1.30); CM-148 submit-time mismatch modal added v1.70.00.</t>
         </is>
       </c>
       <c r="G62" s="1" t="inlineStr">
@@ -3080,7 +3090,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>Decide the engine-profile strategy. Restoration: per-size EXACT sets (less resident VRAM + tuned kernels; current 8GB recommendation) vs a single WIDE set with opt at the common size (note the unused OPT_DYNAMIC_BATCH=60 constant; only preprocess/upsample vary with N - the 4 loop-body engines are batch-1 static and SHARED across sets, so extra sizes are cheap). Measure the off-opt penalty empirically (A/B: MCL 60 via b60 vs b180, compare t_restore). Decide what Manage Models compiles by default and how the resolver + UI constraints present it. Detection: same question for imgsz (640 vs 960 are separate engines). Extends CM-040; ties to CM-061. From CM-049.</t>
+          <t>Decide the engine-profile strategy. Restoration: per-size EXACT sets (less resident VRAM + tuned kernels; current 8GB recommendation) vs a single WIDE set with opt at the common size (note the unused OPT_DYNAMIC_BATCH=60 constant; only preprocess/upsample vary with N - the 4 loop-body engines are batch-1 static and SHARED across sets, so extra sizes are cheap). Measure the off-opt penalty empirically (A/B: MCL 60 via b60 vs b180, compare t_restore). Decide what Manage Models compiles by default and how the resolver + UI constraints present it. Detection: same question for imgsz (640 vs 960 are separate engines). Extends CM-040; ties to CM-061. From CM-049. || UPDATE 2026-09-11: Largely superseded: v1.60 fixed-batch sub-engines serve any Max Clip (CM-104); per-size detection engines remain in CM-151.</t>
         </is>
       </c>
       <c r="G63" s="1" t="inlineStr">
@@ -3136,7 +3146,7 @@
       <c r="I64" s="1" t="n"/>
       <c r="J64" s="1" t="n"/>
     </row>
-    <row r="65" ht="60" customHeight="1">
+    <row r="65" hidden="1" ht="60" customHeight="1">
       <c r="A65" s="1" t="inlineStr">
         <is>
           <t>CM-064</t>
@@ -3476,7 +3486,7 @@
       <c r="I72" s="1" t="n"/>
       <c r="J72" s="1" t="n"/>
     </row>
-    <row r="73" ht="60" customHeight="1">
+    <row r="73" hidden="1" ht="60" customHeight="1">
       <c r="A73" s="1" t="inlineStr">
         <is>
           <t>CM-072</t>
@@ -3560,7 +3570,7 @@
       <c r="I74" s="1" t="n"/>
       <c r="J74" s="1" t="n"/>
     </row>
-    <row r="75" ht="45" customHeight="1">
+    <row r="75" hidden="1" ht="45" customHeight="1">
       <c r="A75" s="1" t="inlineStr">
         <is>
           <t>CM-074</t>
@@ -3573,7 +3583,7 @@
       </c>
       <c r="C75" s="1" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D75" s="1" t="inlineStr">
@@ -3588,7 +3598,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>Viewer assumes equirect-180 LR; fisheye VR sources project wrong. Add a projection dropdown - swap is confined to the direction-&gt;UV function in the fragment shader. Documented as known limitation in v1.10/v1.20 notes.</t>
+          <t>Viewer assumes equirect-180 LR; fisheye VR sources project wrong. Add a projection dropdown - swap is confined to the direction-&gt;UV function in the fragment shader. Documented as known limitation in v1.10/v1.20 notes. || UPDATE 2026-09-11: Shipped as VR Projection selector (Batch 19, v1.30).</t>
         </is>
       </c>
       <c r="G75" s="1" t="inlineStr">
@@ -3602,7 +3612,7 @@
       <c r="I75" s="1" t="n"/>
       <c r="J75" s="1" t="n"/>
     </row>
-    <row r="76" ht="135" customHeight="1">
+    <row r="76" hidden="1" ht="135" customHeight="1">
       <c r="A76" s="1" t="inlineStr">
         <is>
           <t>CM-075</t>
@@ -3644,7 +3654,7 @@
       <c r="I76" s="1" t="n"/>
       <c r="J76" s="1" t="n"/>
     </row>
-    <row r="77">
+    <row r="77" hidden="1" ht="60" customHeight="1">
       <c r="A77" s="1" t="inlineStr">
         <is>
           <t>CM-076</t>
@@ -3686,7 +3696,7 @@
       <c r="I77" s="1" t="n"/>
       <c r="J77" s="1" t="n"/>
     </row>
-    <row r="78">
+    <row r="78" hidden="1" ht="105" customHeight="1">
       <c r="A78" s="1" t="inlineStr">
         <is>
           <t>CM-077</t>
@@ -3728,7 +3738,7 @@
       <c r="I78" s="1" t="n"/>
       <c r="J78" s="1" t="n"/>
     </row>
-    <row r="79">
+    <row r="79" hidden="1" ht="105" customHeight="1">
       <c r="A79" s="1" t="inlineStr">
         <is>
           <t>CM-078</t>
@@ -3770,7 +3780,7 @@
       <c r="I79" s="1" t="n"/>
       <c r="J79" s="1" t="n"/>
     </row>
-    <row r="80">
+    <row r="80" hidden="1" ht="60" customHeight="1">
       <c r="A80" s="1" t="inlineStr">
         <is>
           <t>CM-079</t>
@@ -3812,7 +3822,7 @@
       <c r="I80" s="1" t="n"/>
       <c r="J80" s="1" t="n"/>
     </row>
-    <row r="81">
+    <row r="81" hidden="1" ht="75" customHeight="1">
       <c r="A81" s="1" t="inlineStr">
         <is>
           <t>CM-080</t>
@@ -3854,7 +3864,7 @@
       <c r="I81" s="1" t="n"/>
       <c r="J81" s="1" t="n"/>
     </row>
-    <row r="82">
+    <row r="82" hidden="1" ht="75" customHeight="1">
       <c r="A82" s="1" t="inlineStr">
         <is>
           <t>CM-081</t>
@@ -3896,7 +3906,7 @@
       <c r="I82" s="1" t="n"/>
       <c r="J82" s="1" t="n"/>
     </row>
-    <row r="83">
+    <row r="83" hidden="1" ht="60" customHeight="1">
       <c r="A83" s="1" t="inlineStr">
         <is>
           <t>CM-082</t>
@@ -3938,7 +3948,7 @@
       <c r="I83" s="1" t="n"/>
       <c r="J83" s="1" t="n"/>
     </row>
-    <row r="84">
+    <row r="84" ht="45" customHeight="1">
       <c r="A84" s="1" t="inlineStr">
         <is>
           <t>CM-083</t>
@@ -3946,7 +3956,7 @@
       </c>
       <c r="B84" s="1" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="C84" s="1" t="inlineStr">
@@ -3980,7 +3990,7 @@
       <c r="I84" s="1" t="n"/>
       <c r="J84" s="1" t="n"/>
     </row>
-    <row r="85">
+    <row r="85" hidden="1" ht="75" customHeight="1">
       <c r="A85" s="1" t="inlineStr">
         <is>
           <t>CM-084</t>
@@ -3993,7 +4003,7 @@
       </c>
       <c r="C85" s="1" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D85" s="1" t="inlineStr">
@@ -4008,7 +4018,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>Opt-in host-memory backend for FrameStore to relieve the 8GB VRAM ceiling; Auto decides via the canary's link-generation reading (narrow/Gen1 eGPU links make paging fatal, Gen3+ survives it). Agreed and queued; post-v1.40.</t>
+          <t>Opt-in host-memory backend for FrameStore to relieve the 8GB VRAM ceiling; Auto decides via the canary's link-generation reading (narrow/Gen1 eGPU links make paging fatal, Gen3+ survives it). Agreed and queued; post-v1.40. || UPDATE 2026-09-11: Shipped as Store backend auto/device/host (host store proven on 4K 8GB 09-09). Auto-&gt;host decision rework = CM-175.</t>
         </is>
       </c>
       <c r="G85" s="1" t="inlineStr">
@@ -4022,7 +4032,7 @@
       <c r="I85" s="1" t="n"/>
       <c r="J85" s="1" t="n"/>
     </row>
-    <row r="86">
+    <row r="86" ht="60" customHeight="1">
       <c r="A86" s="1" t="inlineStr">
         <is>
           <t>CM-085</t>
@@ -4064,7 +4074,7 @@
       <c r="I86" s="1" t="n"/>
       <c r="J86" s="1" t="n"/>
     </row>
-    <row r="87">
+    <row r="87" ht="120" customHeight="1">
       <c r="A87" s="1" t="inlineStr">
         <is>
           <t>CM-086</t>
@@ -4092,7 +4102,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>Field report: the FaceFusion (support-mask) blend creates artifacts. Ships in v1.40 release notes as a known issue worded as reported behavior ('some users have reported...'). Investigate create_support_blend_mask alpha vs the legacy rectangular blend. Parked by agreement.</t>
+          <t>Field report: the FaceFusion (support-mask) blend creates artifacts. Ships in v1.40 release notes as a known issue worded as reported behavior ('some users have reported...'). Investigate create_support_blend_mask alpha vs the legacy rectangular blend. Parked by agreement. || UPDATE 2026-09-11: CONFIRMED 09-11 on the 9060 XT: the facefusion (support) blend feathers inward only and adds visible noise/fringe at the paste-back edge; the AMD benchmark rows (6h51m/7h06m) were measured with it. Default stays legacy ('none'); decide: fix the support mask (dilate to the mosaic bleed + outward feather) or drop the option. Presets revert to legacy.</t>
         </is>
       </c>
       <c r="G87" s="1" t="inlineStr">
@@ -4106,7 +4116,7 @@
       <c r="I87" s="1" t="n"/>
       <c r="J87" s="1" t="n"/>
     </row>
-    <row r="88">
+    <row r="88" hidden="1" ht="60" customHeight="1">
       <c r="A88" s="1" t="inlineStr">
         <is>
           <t>CM-087</t>
@@ -4119,7 +4129,7 @@
       </c>
       <c r="C88" s="1" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D88" s="1" t="inlineStr">
@@ -4134,7 +4144,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>Rebuild the packaged exe with Batches 26-29 + watchdog integrated (spec ledger must pass). Clean-machine checks: [Secondary] RTX Super-Res ACTIVE, [TemporalFix] ACTIVE with no manual weight placement, a folder batch run, and -cli.exe live stdout in PowerShell.</t>
+          <t>Rebuild the packaged exe with Batches 26-29 + watchdog integrated (spec ledger must pass). Clean-machine checks: [Secondary] RTX Super-Res ACTIVE, [TemporalFix] ACTIVE with no manual weight placement, a folder batch run, and -cli.exe live stdout in PowerShell. || UPDATE 2026-09-11: v1.40.00 released 2026-07-30.</t>
         </is>
       </c>
       <c r="G88" s="1" t="inlineStr">
@@ -4148,7 +4158,7 @@
       <c r="I88" s="1" t="n"/>
       <c r="J88" s="1" t="n"/>
     </row>
-    <row r="89">
+    <row r="89" hidden="1" ht="75" customHeight="1">
       <c r="A89" s="1" t="inlineStr">
         <is>
           <t>CM-088</t>
@@ -4161,7 +4171,7 @@
       </c>
       <c r="C89" s="1" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D89" s="1" t="inlineStr">
@@ -4176,7 +4186,7 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>README + release notes + forum BBCode; SFW text/UI screenshots only. Must include: the 8GB law (MCL 60 + preset P5), recommended preset (scaler on, temporal stability on), -cli.exe, three-file installer download, two-pass censoring, max-recall preset, known issues (FaceFusion blend artifacts; Quest seek guidance pending CM-089).</t>
+          <t>README + release notes + forum BBCode; SFW text/UI screenshots only. Must include: the 8GB law (MCL 60 + preset P5), recommended preset (scaler on, temporal stability on), -cli.exe, three-file installer download, two-pass censoring, max-recall preset, known issues (FaceFusion blend artifacts; Quest seek guidance pending CM-089). || UPDATE 2026-09-11: v1.40.00 docs shipped 2026-07-30.</t>
         </is>
       </c>
       <c r="G89" s="1" t="inlineStr">
@@ -4190,7 +4200,7 @@
       <c r="I89" s="1" t="n"/>
       <c r="J89" s="1" t="n"/>
     </row>
-    <row r="90">
+    <row r="90" ht="45" customHeight="1">
       <c r="A90" s="1" t="inlineStr">
         <is>
           <t>CM-089</t>
@@ -4232,7 +4242,7 @@
       <c r="I90" s="1" t="n"/>
       <c r="J90" s="1" t="n"/>
     </row>
-    <row r="91">
+    <row r="91" hidden="1" ht="75" customHeight="1">
       <c r="A91" s="1" t="inlineStr">
         <is>
           <t>CM-090</t>
@@ -4245,7 +4255,7 @@
       </c>
       <c r="C91" s="1" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D91" s="1" t="inlineStr">
@@ -4260,7 +4270,7 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>CORRECTED 2026-07-28: the completion modal DOES keep the elapsed time (earlier report was mistaken). Remaining ask: add an elapsed-time display to the Preview and Test Frame flows too, so every kind of run reports how long it took. Low priority; next time the UI is touched.</t>
+          <t>CORRECTED 2026-07-28: the completion modal DOES keep the elapsed time (earlier report was mistaken). Remaining ask: add an elapsed-time display to the Preview and Test Frame flows too, so every kind of run reports how long it took. Low priority; next time the UI is touched. || UPDATE 2026-09-11: Shipped: elapsed clocks on Preview/Test Frame (T9b _wireElapsedClocks, v1.70.00).</t>
         </is>
       </c>
       <c r="G91" s="1" t="inlineStr">
@@ -4274,8 +4284,3192 @@
       <c r="I91" s="1" t="n"/>
       <c r="J91" s="1" t="n"/>
     </row>
+    <row r="92" hidden="1" ht="30" customHeight="1">
+      <c r="A92" s="1" t="inlineStr">
+        <is>
+          <t>CM-091</t>
+        </is>
+      </c>
+      <c r="B92" s="1" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C92" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D92" s="1" t="inlineStr">
+        <is>
+          <t>Encode</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>AV1 seek fix: repeated sequence headers at remux</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>NVENC AV1 omits repeated seq headers; encoder self-heals the IVF stream at remux. v1.40.00 (Batch 30b).</t>
+        </is>
+      </c>
+      <c r="G92" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="H92" s="3" t="n">
+        <v>46232</v>
+      </c>
+      <c r="I92" s="1" t="n"/>
+      <c r="J92" s="1" t="n"/>
+    </row>
+    <row r="93" hidden="1" ht="30" customHeight="1">
+      <c r="A93" s="1" t="inlineStr">
+        <is>
+          <t>CM-093</t>
+        </is>
+      </c>
+      <c r="B93" s="1" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C93" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D93" s="1" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>Intel Arc (XPU) edition, Phase 0</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>XPU device path, ffmpeg/QSV decode lane, CM_HW_DECODE env switch. Shipped as ChitraMaya-Intel-ARC v1.41.</t>
+        </is>
+      </c>
+      <c r="G93" s="1" t="inlineStr">
+        <is>
+          <t>Gman + Claude</t>
+        </is>
+      </c>
+      <c r="H93" s="3" t="n">
+        <v>46242</v>
+      </c>
+      <c r="I93" s="1" t="n"/>
+      <c r="J93" s="1" t="n"/>
+    </row>
+    <row r="94" hidden="1" ht="30" customHeight="1">
+      <c r="A94" s="1" t="inlineStr">
+        <is>
+          <t>CM-095</t>
+        </is>
+      </c>
+      <c r="B94" s="1" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C94" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D94" s="1" t="inlineStr">
+        <is>
+          <t>Mosaic</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>Checkpoint load error message (which file / why / what to do)</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>Wrong or corrupt .pth surfaces as one plain message instead of a pickle traceback. v1.50.00. CM-181 extends it for the lada _full training checkpoint (mmengine).</t>
+        </is>
+      </c>
+      <c r="G94" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="H94" s="3" t="n">
+        <v>46244</v>
+      </c>
+      <c r="I94" s="1" t="n"/>
+      <c r="J94" s="1" t="n"/>
+    </row>
+    <row r="95" hidden="1" ht="30" customHeight="1">
+      <c r="A95" s="1" t="inlineStr">
+        <is>
+          <t>CM-104</t>
+        </is>
+      </c>
+      <c r="B95" s="1" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C95" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D95" s="1" t="inlineStr">
+        <is>
+          <t>Mosaic</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>Fixed-batch BasicVSR++ sub-engine set (any Max Clip)</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>One memory-lean compiled set serves every Max Clip; legacy clip-sized sets still load. v1.60.00.</t>
+        </is>
+      </c>
+      <c r="G95" s="1" t="inlineStr">
+        <is>
+          <t>Claude Analysis</t>
+        </is>
+      </c>
+      <c r="H95" s="3" t="n">
+        <v>46252</v>
+      </c>
+      <c r="I95" s="1" t="n"/>
+      <c r="J95" s="1" t="n"/>
+    </row>
+    <row r="96" hidden="1" ht="30" customHeight="1">
+      <c r="A96" s="1" t="inlineStr">
+        <is>
+          <t>CM-105</t>
+        </is>
+      </c>
+      <c r="B96" s="1" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C96" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D96" s="1" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>AMD ROCm edition probe + first builds</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>ROCm torch flavour asserted in spec; three venvs one tree. Shipped as ChitraMaya-AMD-ROCM (1.40.02 -&gt; 1.61 -&gt; 1.70).</t>
+        </is>
+      </c>
+      <c r="G96" s="1" t="inlineStr">
+        <is>
+          <t>Gman + Claude</t>
+        </is>
+      </c>
+      <c r="H96" s="3" t="n">
+        <v>46246</v>
+      </c>
+      <c r="I96" s="1" t="n"/>
+      <c r="J96" s="1" t="n"/>
+    </row>
+    <row r="97" hidden="1">
+      <c r="A97" s="1" t="inlineStr">
+        <is>
+          <t>CM-109</t>
+        </is>
+      </c>
+      <c r="B97" s="1" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C97" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D97" s="1" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>Copy button on the compile log</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>Standing rule: every log pane has Copy. v1.50 (Batch 50).</t>
+        </is>
+      </c>
+      <c r="G97" s="1" t="inlineStr">
+        <is>
+          <t>Gman request</t>
+        </is>
+      </c>
+      <c r="H97" s="3" t="n">
+        <v>46246</v>
+      </c>
+      <c r="I97" s="1" t="n"/>
+      <c r="J97" s="1" t="n"/>
+    </row>
+    <row r="98" hidden="1" ht="105" customHeight="1">
+      <c r="A98" s="1" t="inlineStr">
+        <is>
+          <t>CM-112</t>
+        </is>
+      </c>
+      <c r="B98" s="1" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C98" s="1" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="D98" s="1" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>Training framework (Phase A detection PoC -&gt; B -&gt; C restoration fine-tune -&gt; D model hub)</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>Phase A/A2 detection loop proven in the frozen app; Panels 1-2 shipped hidden behind trainingUI key (v1.70.00); Phase C: recipe v1 -&gt; ft_v0/ft_v1 trained and examined; **ft_v1 CONFIRMED 09-11 to invent structure on real studio mosaic (domain mismatch: region-proportional ROI-anchored block vs studio block fixed in screen space 2.0-2.4% H; 720p GT softness) -&gt; OUT of every standard config; recipe v2 + ft_v2 next; exam rule: watch a full studio-mosaic restoration vs generic before any model leaves the lab.** Phase D hub spec written. Splash release after Panel 3.</t>
+        </is>
+      </c>
+      <c r="G98" s="1" t="inlineStr">
+        <is>
+          <t>Gman + Claude</t>
+        </is>
+      </c>
+      <c r="H98" s="3" t="n">
+        <v>46256</v>
+      </c>
+      <c r="I98" s="1" t="n"/>
+      <c r="J98" s="1" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="1" t="inlineStr">
+        <is>
+          <t>CM-114</t>
+        </is>
+      </c>
+      <c r="B99" s="1" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C99" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D99" s="1" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t>Save segment preview</t>
+        </is>
+      </c>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>Save the segment preview output as a file.</t>
+        </is>
+      </c>
+      <c r="G99" s="1" t="inlineStr">
+        <is>
+          <t>Gman request</t>
+        </is>
+      </c>
+      <c r="H99" s="3" t="n">
+        <v>46259</v>
+      </c>
+      <c r="I99" s="1" t="n"/>
+      <c r="J99" s="1" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="1" t="inlineStr">
+        <is>
+          <t>CM-119</t>
+        </is>
+      </c>
+      <c r="B100" s="1" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C100" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D100" s="1" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>Restore button dead on an anchored range</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>Reported 08-30; verify on 1.70.00 before fixing.</t>
+        </is>
+      </c>
+      <c r="G100" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="H100" s="3" t="n">
+        <v>46264</v>
+      </c>
+      <c r="I100" s="1" t="n"/>
+      <c r="J100" s="1" t="n"/>
+    </row>
+    <row r="101" hidden="1" ht="30" customHeight="1">
+      <c r="A101" s="1" t="inlineStr">
+        <is>
+          <t>CM-120</t>
+        </is>
+      </c>
+      <c r="B101" s="1" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C101" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D101" s="1" t="inlineStr">
+        <is>
+          <t>Encode</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>TS remux candidates -&gt; Temp folder</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>Temp remux beside the source failed on drive F:; candidates now [Temp, src.parent] with free-space check. v1.70.00 (T9b).</t>
+        </is>
+      </c>
+      <c r="G101" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="H101" s="3" t="n">
+        <v>46267</v>
+      </c>
+      <c r="I101" s="1" t="n"/>
+      <c r="J101" s="1" t="n"/>
+    </row>
+    <row r="102" hidden="1" ht="30" customHeight="1">
+      <c r="A102" s="1" t="inlineStr">
+        <is>
+          <t>CM-124</t>
+        </is>
+      </c>
+      <c r="B102" s="1" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C102" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D102" s="1" t="inlineStr">
+        <is>
+          <t>Encode</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>Progress-supervised finalize (disk-progress watchdog)</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>Remux supervised by output size growth, size-scaled timeout, 600 s no-growth kill. v1.61.00. See CM-174/CM-179/CM-187 for what it misreads.</t>
+        </is>
+      </c>
+      <c r="G102" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="H102" s="3" t="n">
+        <v>46261</v>
+      </c>
+      <c r="I102" s="1" t="n"/>
+      <c r="J102" s="1" t="n"/>
+    </row>
+    <row r="103" hidden="1">
+      <c r="A103" s="1" t="inlineStr">
+        <is>
+          <t>CM-125</t>
+        </is>
+      </c>
+      <c r="B103" s="1" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C103" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D103" s="1" t="inlineStr">
+        <is>
+          <t>Encode</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>Remux .part output + discard on failure</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>Half-written outputs never look finished. v1.61.00.</t>
+        </is>
+      </c>
+      <c r="G103" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="H103" s="3" t="n">
+        <v>46261</v>
+      </c>
+      <c r="I103" s="1" t="n"/>
+      <c r="J103" s="1" t="n"/>
+    </row>
+    <row r="104" hidden="1">
+      <c r="A104" s="1" t="inlineStr">
+        <is>
+          <t>CM-126</t>
+        </is>
+      </c>
+      <c r="B104" s="1" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C104" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D104" s="1" t="inlineStr">
+        <is>
+          <t>Packaging</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>Single-file installer fold-back for AMD/Intel</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>ChitraMaya-rocm-install.exe / ChitraMaya-xpu-install.exe. v1.61.00.</t>
+        </is>
+      </c>
+      <c r="G104" s="1" t="inlineStr">
+        <is>
+          <t>Gman + Claude</t>
+        </is>
+      </c>
+      <c r="H104" s="3" t="n">
+        <v>46262</v>
+      </c>
+      <c r="I104" s="1" t="n"/>
+      <c r="J104" s="1" t="n"/>
+    </row>
+    <row r="105" hidden="1" ht="30" customHeight="1">
+      <c r="A105" s="1" t="inlineStr">
+        <is>
+          <t>CM-127</t>
+        </is>
+      </c>
+      <c r="B105" s="1" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C105" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D105" s="1" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t>Long filenames (MAX_PATH) hardening</t>
+        </is>
+      </c>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>Stem-free probe, hashed remux-cache name, shortened sidecars, clear refusal &gt;259. v1.70.00.</t>
+        </is>
+      </c>
+      <c r="G105" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="H105" s="3" t="n">
+        <v>46263</v>
+      </c>
+      <c r="I105" s="1" t="n"/>
+      <c r="J105" s="1" t="n"/>
+    </row>
+    <row r="106" hidden="1" ht="30" customHeight="1">
+      <c r="A106" s="1" t="inlineStr">
+        <is>
+          <t>CM-128</t>
+        </is>
+      </c>
+      <c r="B106" s="1" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C106" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D106" s="1" t="inlineStr">
+        <is>
+          <t>Mosaic</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>Unified-memory exhaustion: restore window split-retry</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>XPU + &lt;20 GB RAM -&gt; 96-frame windows; out-of-resources retries as halves. v1.61.00 (Batch 62).</t>
+        </is>
+      </c>
+      <c r="G106" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="H106" s="3" t="n">
+        <v>46264</v>
+      </c>
+      <c r="I106" s="1" t="n"/>
+      <c r="J106" s="1" t="n"/>
+    </row>
+    <row r="107" ht="30" customHeight="1">
+      <c r="A107" s="1" t="inlineStr">
+        <is>
+          <t>CM-129</t>
+        </is>
+      </c>
+      <c r="B107" s="1" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C107" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D107" s="1" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>Zero-frame run must self-grade as failure</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>A run that delivered 0 frames ended status=complete. Fold into CM-153 (restored==0 handling) and CM-177 (decoder frame-count sanity).</t>
+        </is>
+      </c>
+      <c r="G107" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="H107" s="3" t="n">
+        <v>46264</v>
+      </c>
+      <c r="I107" s="1" t="n"/>
+      <c r="J107" s="1" t="n"/>
+    </row>
+    <row r="108" ht="30" customHeight="1">
+      <c r="A108" s="1" t="inlineStr">
+        <is>
+          <t>CM-130</t>
+        </is>
+      </c>
+      <c r="B108" s="1" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C108" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D108" s="1" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>In-app player: HEVC extension missing -&gt; silent black</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>Detect onerror and show the install-extension message. README known-issue line shipped.</t>
+        </is>
+      </c>
+      <c r="G108" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="H108" s="3" t="n">
+        <v>46264</v>
+      </c>
+      <c r="I108" s="1" t="n"/>
+      <c r="J108" s="1" t="n"/>
+    </row>
+    <row r="109" hidden="1" ht="30" customHeight="1">
+      <c r="A109" s="1" t="inlineStr">
+        <is>
+          <t>CM-131</t>
+        </is>
+      </c>
+      <c r="B109" s="1" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C109" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D109" s="1" t="inlineStr">
+        <is>
+          <t>Packaging</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>ffmpeg 9 compatibility (-vsync removed) + spec version gate</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>-fps_mode passthrough; spec refuses unknown majors and mixed pairs; majors {8,9}. v1.61.00 (Batches 63-65).</t>
+        </is>
+      </c>
+      <c r="G109" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="H109" s="3" t="n">
+        <v>46264</v>
+      </c>
+      <c r="I109" s="1" t="n"/>
+      <c r="J109" s="1" t="n"/>
+    </row>
+    <row r="110" hidden="1">
+      <c r="A110" s="1" t="inlineStr">
+        <is>
+          <t>CM-132</t>
+        </is>
+      </c>
+      <c r="B110" s="1" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C110" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D110" s="1" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>Self-check names the matching edition when the GPU vendor is wrong</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>CLI text. v1.70.00. Message-box version = CM-163.</t>
+        </is>
+      </c>
+      <c r="G110" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="H110" s="3" t="n">
+        <v>46266</v>
+      </c>
+      <c r="I110" s="1" t="n"/>
+      <c r="J110" s="1" t="n"/>
+    </row>
+    <row r="111" hidden="1">
+      <c r="A111" s="1" t="inlineStr">
+        <is>
+          <t>CM-136</t>
+        </is>
+      </c>
+      <c r="B111" s="1" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C111" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D111" s="1" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr">
+        <is>
+          <t>SHA-256 table on release pages</t>
+        </is>
+      </c>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>Public commitment (lada Codeberg thread) closed with the 1.70.00 release pages.</t>
+        </is>
+      </c>
+      <c r="G111" s="1" t="inlineStr">
+        <is>
+          <t>Gman + Claude</t>
+        </is>
+      </c>
+      <c r="H111" s="3" t="n">
+        <v>46266</v>
+      </c>
+      <c r="I111" s="1" t="n"/>
+      <c r="J111" s="1" t="n"/>
+    </row>
+    <row r="112" hidden="1" ht="45" customHeight="1">
+      <c r="A112" s="1" t="inlineStr">
+        <is>
+          <t>CM-139</t>
+        </is>
+      </c>
+      <c r="B112" s="1" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C112" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D112" s="1" t="inlineStr">
+        <is>
+          <t>Mosaic</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t>Real-ESRGAN 4x secondary (all editions)</t>
+        </is>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>realesr-general-x4v3, plain torch, bundled weights. v1.70.00 (Batch 68). 09-11: cleared as the source of the 'generative' artifacts (that was ft_v1, CM-112); the ESRGAN-on run is the pending AMD quality check.</t>
+        </is>
+      </c>
+      <c r="G112" s="1" t="inlineStr">
+        <is>
+          <t>Gman + Claude</t>
+        </is>
+      </c>
+      <c r="H112" s="3" t="n">
+        <v>46267</v>
+      </c>
+      <c r="I112" s="1" t="n"/>
+      <c r="J112" s="1" t="n"/>
+    </row>
+    <row r="113" hidden="1">
+      <c r="A113" s="1" t="inlineStr">
+        <is>
+          <t>CM-141</t>
+        </is>
+      </c>
+      <c r="B113" s="1" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C113" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D113" s="1" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="E113" s="2" t="inlineStr">
+        <is>
+          <t>YOLO_AUTOINSTALL=false at entry</t>
+        </is>
+      </c>
+      <c r="F113" s="2" t="inlineStr">
+        <is>
+          <t>No pip at runtime inside the frozen app. v1.70.00 (Batch 79).</t>
+        </is>
+      </c>
+      <c r="G113" s="1" t="inlineStr">
+        <is>
+          <t>Claude Analysis</t>
+        </is>
+      </c>
+      <c r="H113" s="3" t="n">
+        <v>46267</v>
+      </c>
+      <c r="I113" s="1" t="n"/>
+      <c r="J113" s="1" t="n"/>
+    </row>
+    <row r="114" ht="45" customHeight="1">
+      <c r="A114" s="1" t="inlineStr">
+        <is>
+          <t>CM-142</t>
+        </is>
+      </c>
+      <c r="B114" s="1" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C114" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D114" s="1" t="inlineStr">
+        <is>
+          <t>Decode</t>
+        </is>
+      </c>
+      <c r="E114" s="2" t="inlineStr">
+        <is>
+          <t>ffmpeg/QSV decode lane: per-frame PTS capture</t>
+        </is>
+      </c>
+      <c r="F114" s="2" t="inlineStr">
+        <is>
+          <t>128 frames dropped unlocatable on one source family (no PTS on the pipe lane); NVDEC lane gap-filled the same drops. Fix shape: PTS capture on the ffmpeg lane. Relevant to CM-171 transport rework.</t>
+        </is>
+      </c>
+      <c r="G114" s="1" t="inlineStr">
+        <is>
+          <t>Claude Analysis</t>
+        </is>
+      </c>
+      <c r="H114" s="3" t="n">
+        <v>46266</v>
+      </c>
+      <c r="I114" s="1" t="n"/>
+      <c r="J114" s="1" t="n"/>
+    </row>
+    <row r="115" hidden="1" ht="45" customHeight="1">
+      <c r="A115" s="1" t="inlineStr">
+        <is>
+          <t>CM-146</t>
+        </is>
+      </c>
+      <c r="B115" s="1" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C115" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D115" s="1" t="inlineStr">
+        <is>
+          <t>Mosaic</t>
+        </is>
+      </c>
+      <c r="E115" s="2" t="inlineStr">
+        <is>
+          <t>Secondary denoise wiring (the missed last hop)</t>
+        </is>
+      </c>
+      <c r="F115" s="2" t="inlineStr">
+        <is>
+          <t>secondary_denoise now reaches the pipeline; every earlier denoise A/B had run denoise=none. v1.70.00 (Batch 74). Verdict since: ultra = no visible change at +60% restore time; default none.</t>
+        </is>
+      </c>
+      <c r="G115" s="1" t="inlineStr">
+        <is>
+          <t>Claude Analysis</t>
+        </is>
+      </c>
+      <c r="H115" s="3" t="n">
+        <v>46267</v>
+      </c>
+      <c r="I115" s="1" t="n"/>
+      <c r="J115" s="1" t="n"/>
+    </row>
+    <row r="116" hidden="1">
+      <c r="A116" s="1" t="inlineStr">
+        <is>
+          <t>CM-148</t>
+        </is>
+      </c>
+      <c r="B116" s="1" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C116" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D116" s="1" t="inlineStr">
+        <is>
+          <t>Detection</t>
+        </is>
+      </c>
+      <c r="E116" s="2" t="inlineStr">
+        <is>
+          <t>Engine imgsz mismatch: submit-time modal</t>
+        </is>
+      </c>
+      <c r="F116" s="2" t="inlineStr">
+        <is>
+          <t>Use engine size / Continue on PyTorch / Manage Models. v1.70.00 (Batch 76).</t>
+        </is>
+      </c>
+      <c r="G116" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="H116" s="3" t="n">
+        <v>46267</v>
+      </c>
+      <c r="I116" s="1" t="n"/>
+      <c r="J116" s="1" t="n"/>
+    </row>
+    <row r="117" ht="30" customHeight="1">
+      <c r="A117" s="1" t="inlineStr">
+        <is>
+          <t>CM-149</t>
+        </is>
+      </c>
+      <c r="B117" s="1" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C117" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D117" s="1" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="E117" s="2" t="inlineStr">
+        <is>
+          <t>cudaExpandableSegments key REWORK</t>
+        </is>
+      </c>
+      <c r="F117" s="2" t="inlineStr">
+        <is>
+          <t>expandable_segments unsupported by PyTorch on Windows; map the key to max_split_size_mb / garbage_collection_threshold with an honest print.</t>
+        </is>
+      </c>
+      <c r="G117" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="H117" s="3" t="n">
+        <v>46267</v>
+      </c>
+      <c r="I117" s="1" t="n"/>
+      <c r="J117" s="1" t="n"/>
+    </row>
+    <row r="118" ht="30" customHeight="1">
+      <c r="A118" s="1" t="inlineStr">
+        <is>
+          <t>CM-150</t>
+        </is>
+      </c>
+      <c r="B118" s="1" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C118" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D118" s="1" t="inlineStr">
+        <is>
+          <t>Decode</t>
+        </is>
+      </c>
+      <c r="E118" s="2" t="inlineStr">
+        <is>
+          <t>TS-in-MKV sources: fallback path</t>
+        </is>
+      </c>
+      <c r="F118" s="2" t="inlineStr">
+        <is>
+          <t>Fallback reproduced flawless on all five TS mkvs both nights; decide whether to keep as-is or make the primary path handle them.</t>
+        </is>
+      </c>
+      <c r="G118" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="H118" s="3" t="n">
+        <v>46267</v>
+      </c>
+      <c r="I118" s="1" t="n"/>
+      <c r="J118" s="1" t="n"/>
+    </row>
+    <row r="119" ht="60" customHeight="1">
+      <c r="A119" s="1" t="inlineStr">
+        <is>
+          <t>CM-151</t>
+        </is>
+      </c>
+      <c r="B119" s="1" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C119" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D119" s="1" t="inlineStr">
+        <is>
+          <t>Detection</t>
+        </is>
+      </c>
+      <c r="E119" s="2" t="inlineStr">
+        <is>
+          <t>Engine manifest + 'Compiled (with warnings)' badge + surfaced fallback</t>
+        </is>
+      </c>
+      <c r="F119" s="2" t="inlineStr">
+        <is>
+          <t>Sidecar per engine: source hash/size, compile params incl. dynamic range, GPU/CC/TRT/torch/driver/build stamp, TRT OOM/tactic-skip counts. Badge says degraded builds; run reports PyTorch fallback; per-size engines + dynamic-range default in the mismatch modal. Driven by GitHub issue #7 (RTX 3050 4 GB). NEXT DROP.</t>
+        </is>
+      </c>
+      <c r="G119" s="1" t="inlineStr">
+        <is>
+          <t>GitHub issue #7</t>
+        </is>
+      </c>
+      <c r="H119" s="3" t="n">
+        <v>46268</v>
+      </c>
+      <c r="I119" s="1" t="n"/>
+      <c r="J119" s="1" t="inlineStr">
+        <is>
+          <t>https://github.com/seatv/ChitraMaya/issues/7</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="30" customHeight="1">
+      <c r="A120" s="1" t="inlineStr">
+        <is>
+          <t>CM-152</t>
+        </is>
+      </c>
+      <c r="B120" s="1" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C120" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D120" s="1" t="inlineStr">
+        <is>
+          <t>Mosaic</t>
+        </is>
+      </c>
+      <c r="E120" s="2" t="inlineStr">
+        <is>
+          <t>Honest miss accounting</t>
+        </is>
+      </c>
+      <c r="F120" s="2" t="inlineStr">
+        <is>
+          <t>Rename visible_miss -&gt; clip_gap_frames; passthrough audit with a second-opinion detector labelled ESTIMATE.</t>
+        </is>
+      </c>
+      <c r="G120" s="1" t="inlineStr">
+        <is>
+          <t>Claude Analysis</t>
+        </is>
+      </c>
+      <c r="H120" s="3" t="n">
+        <v>46269</v>
+      </c>
+      <c r="I120" s="1" t="n"/>
+      <c r="J120" s="1" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="1" t="inlineStr">
+        <is>
+          <t>CM-153</t>
+        </is>
+      </c>
+      <c r="B121" s="1" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C121" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D121" s="1" t="inlineStr">
+        <is>
+          <t>Encode</t>
+        </is>
+      </c>
+      <c r="E121" s="2" t="inlineStr">
+        <is>
+          <t>restored==0 -&gt; lossless copy / 'No mosaic found'</t>
+        </is>
+      </c>
+      <c r="F121" s="2" t="inlineStr">
+        <is>
+          <t>Exactly zero restorations: -c copy remux and say so. Absorbs CM-129.</t>
+        </is>
+      </c>
+      <c r="G121" s="1" t="inlineStr">
+        <is>
+          <t>Claude Analysis</t>
+        </is>
+      </c>
+      <c r="H121" s="3" t="n">
+        <v>46269</v>
+      </c>
+      <c r="I121" s="1" t="n"/>
+      <c r="J121" s="1" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="1" t="inlineStr">
+        <is>
+          <t>CM-154</t>
+        </is>
+      </c>
+      <c r="B122" s="1" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C122" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D122" s="1" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="E122" s="2" t="inlineStr">
+        <is>
+          <t>Detector exam tool</t>
+        </is>
+      </c>
+      <c r="F122" s="2" t="inlineStr">
+        <is>
+          <t>Answer-key scoring against a censor run's report; disagreement sets between detectors.</t>
+        </is>
+      </c>
+      <c r="G122" s="1" t="inlineStr">
+        <is>
+          <t>Claude Analysis</t>
+        </is>
+      </c>
+      <c r="H122" s="3" t="n">
+        <v>46269</v>
+      </c>
+      <c r="I122" s="1" t="n"/>
+      <c r="J122" s="1" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="1" t="inlineStr">
+        <is>
+          <t>CM-155</t>
+        </is>
+      </c>
+      <c r="B123" s="1" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C123" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D123" s="1" t="inlineStr">
+        <is>
+          <t>Mosaic</t>
+        </is>
+      </c>
+      <c r="E123" s="2" t="inlineStr">
+        <is>
+          <t>Planner auto-clamp (Max Clip fitted to VRAM/RAM, announced)</t>
+        </is>
+      </c>
+      <c r="F123" s="2" t="inlineStr">
+        <is>
+          <t>The OCuLink 8 GB@4K case and the AMD MCL-180 case. CM-175 folds in.</t>
+        </is>
+      </c>
+      <c r="G123" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="H123" s="3" t="n">
+        <v>46269</v>
+      </c>
+      <c r="I123" s="1" t="n"/>
+      <c r="J123" s="1" t="n"/>
+    </row>
+    <row r="124" ht="45" customHeight="1">
+      <c r="A124" s="1" t="inlineStr">
+        <is>
+          <t>CM-156</t>
+        </is>
+      </c>
+      <c r="B124" s="1" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C124" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D124" s="1" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="E124" s="2" t="inlineStr">
+        <is>
+          <t>Nits bundle</t>
+        </is>
+      </c>
+      <c r="F124" s="2" t="inlineStr">
+        <is>
+          <t>Detection-rate line in summary/progress modal; cancel-at-zero-frames litter; PCIe canary baseline label; encoder remux stderr utf-8; nvGPUMonitor python_rss for frozen exe; Free-VRAM button / fresh process per VRAM row.</t>
+        </is>
+      </c>
+      <c r="G124" s="1" t="inlineStr">
+        <is>
+          <t>Claude Analysis</t>
+        </is>
+      </c>
+      <c r="H124" s="3" t="n">
+        <v>46269</v>
+      </c>
+      <c r="I124" s="1" t="n"/>
+      <c r="J124" s="1" t="n"/>
+    </row>
+    <row r="125" ht="30" customHeight="1">
+      <c r="A125" s="1" t="inlineStr">
+        <is>
+          <t>CM-157</t>
+        </is>
+      </c>
+      <c r="B125" s="1" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C125" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D125" s="1" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="E125" s="2" t="inlineStr">
+        <is>
+          <t>Compile failure hygiene</t>
+        </is>
+      </c>
+      <c r="F125" s="2" t="inlineStr">
+        <is>
+          <t>[compile] FAILED with likely cause instead of PyInstaller's 'Unhandled exception' dialog (forum screenshots 09-06).</t>
+        </is>
+      </c>
+      <c r="G125" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="H125" s="3" t="n">
+        <v>46271</v>
+      </c>
+      <c r="I125" s="1" t="n"/>
+      <c r="J125" s="1" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="1" t="inlineStr">
+        <is>
+          <t>CM-158</t>
+        </is>
+      </c>
+      <c r="B126" s="1" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C126" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D126" s="1" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="E126" s="2" t="inlineStr">
+        <is>
+          <t>Model hub: safetensors only</t>
+        </is>
+      </c>
+      <c r="F126" s="2" t="inlineStr">
+        <is>
+          <t>Community models distributed as safetensors; no pickle. Phase D spec.</t>
+        </is>
+      </c>
+      <c r="G126" s="1" t="inlineStr">
+        <is>
+          <t>Claude Analysis</t>
+        </is>
+      </c>
+      <c r="H126" s="3" t="n">
+        <v>46271</v>
+      </c>
+      <c r="I126" s="1" t="n"/>
+      <c r="J126" s="1" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="1" t="inlineStr">
+        <is>
+          <t>CM-159</t>
+        </is>
+      </c>
+      <c r="B127" s="1" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C127" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D127" s="1" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="E127" s="2" t="inlineStr">
+        <is>
+          <t>Model hub: ONNX detectors, not .pt</t>
+        </is>
+      </c>
+      <c r="F127" s="2" t="inlineStr">
+        <is>
+          <t>Detectors published as ONNX. Phase D spec.</t>
+        </is>
+      </c>
+      <c r="G127" s="1" t="inlineStr">
+        <is>
+          <t>Claude Analysis</t>
+        </is>
+      </c>
+      <c r="H127" s="3" t="n">
+        <v>46271</v>
+      </c>
+      <c r="I127" s="1" t="n"/>
+      <c r="J127" s="1" t="n"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="1" t="inlineStr">
+        <is>
+          <t>CM-160</t>
+        </is>
+      </c>
+      <c r="B128" s="1" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C128" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D128" s="1" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="E128" s="2" t="inlineStr">
+        <is>
+          <t>Model hub: in-app fetch + hash verify</t>
+        </is>
+      </c>
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t>models.json registry as hash authority; PR-based review. Phase D spec.</t>
+        </is>
+      </c>
+      <c r="G128" s="1" t="inlineStr">
+        <is>
+          <t>Claude Analysis</t>
+        </is>
+      </c>
+      <c r="H128" s="3" t="n">
+        <v>46271</v>
+      </c>
+      <c r="I128" s="1" t="n"/>
+      <c r="J128" s="1" t="n"/>
+    </row>
+    <row r="129" hidden="1">
+      <c r="A129" s="1" t="inlineStr">
+        <is>
+          <t>CM-161</t>
+        </is>
+      </c>
+      <c r="B129" s="1" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C129" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D129" s="1" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="E129" s="2" t="inlineStr">
+        <is>
+          <t>Edition label in window title and banner</t>
+        </is>
+      </c>
+      <c r="F129" s="2" t="inlineStr">
+        <is>
+          <t>'ChitraMaya 1.70.00 -- AMD edition'. v1.70.00 (T9b).</t>
+        </is>
+      </c>
+      <c r="G129" s="1" t="inlineStr">
+        <is>
+          <t>Gman request</t>
+        </is>
+      </c>
+      <c r="H129" s="3" t="n">
+        <v>46272</v>
+      </c>
+      <c r="I129" s="1" t="n"/>
+      <c r="J129" s="1" t="n"/>
+    </row>
+    <row r="130" hidden="1" ht="30" customHeight="1">
+      <c r="A130" s="1" t="inlineStr">
+        <is>
+          <t>CM-162</t>
+        </is>
+      </c>
+      <c r="B130" s="1" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C130" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D130" s="1" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="E130" s="2" t="inlineStr">
+        <is>
+          <t>README AMD section from in-house testing</t>
+        </is>
+      </c>
+      <c r="F130" s="2" t="inlineStr">
+        <is>
+          <t>Rewritten against measured numbers (T8b/T9h). 09-11: needs the Restoration-FP16 / facefusion / ft_v1 corrections once the ESRGAN-on run is watched.</t>
+        </is>
+      </c>
+      <c r="G130" s="1" t="inlineStr">
+        <is>
+          <t>Gman + Claude</t>
+        </is>
+      </c>
+      <c r="H130" s="3" t="n">
+        <v>46272</v>
+      </c>
+      <c r="I130" s="1" t="n"/>
+      <c r="J130" s="1" t="n"/>
+    </row>
+    <row r="131" hidden="1" ht="30" customHeight="1">
+      <c r="A131" s="1" t="inlineStr">
+        <is>
+          <t>CM-163</t>
+        </is>
+      </c>
+      <c r="B131" s="1" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C131" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D131" s="1" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="E131" s="2" t="inlineStr">
+        <is>
+          <t>GPU gate before the window opens (wrong-edition message box)</t>
+        </is>
+      </c>
+      <c r="F131" s="2" t="inlineStr">
+        <is>
+          <t>Child-process device probe before torch; MessageBoxW naming the GPUs and the matching edition; exit 3; .gpu-gate-ok cache. v1.70.00 (T9c-2).</t>
+        </is>
+      </c>
+      <c r="G131" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="H131" s="3" t="n">
+        <v>46272</v>
+      </c>
+      <c r="I131" s="1" t="n"/>
+      <c r="J131" s="1" t="n"/>
+    </row>
+    <row r="132" hidden="1">
+      <c r="A132" s="1" t="inlineStr">
+        <is>
+          <t>CM-164</t>
+        </is>
+      </c>
+      <c r="B132" s="1" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C132" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D132" s="1" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="E132" s="2" t="inlineStr">
+        <is>
+          <t>TRT toggles hidden on non-CUDA editions</t>
+        </is>
+      </c>
+      <c r="F132" s="2" t="inlineStr">
+        <is>
+          <t>data-edition gate. v1.70.00 (T9b). The scaler dropdown was missed -&gt; CM-184.</t>
+        </is>
+      </c>
+      <c r="G132" s="1" t="inlineStr">
+        <is>
+          <t>Gman request</t>
+        </is>
+      </c>
+      <c r="H132" s="3" t="n">
+        <v>46272</v>
+      </c>
+      <c r="I132" s="1" t="n"/>
+      <c r="J132" s="1" t="n"/>
+    </row>
+    <row r="133" hidden="1">
+      <c r="A133" s="1" t="inlineStr">
+        <is>
+          <t>CM-165</t>
+        </is>
+      </c>
+      <c r="B133" s="1" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C133" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D133" s="1" t="inlineStr">
+        <is>
+          <t>Packaging</t>
+        </is>
+      </c>
+      <c r="E133" s="2" t="inlineStr">
+        <is>
+          <t>.cmd launchers capture ERRORLEVEL and pause with guidance</t>
+        </is>
+      </c>
+      <c r="F133" s="2" t="inlineStr">
+        <is>
+          <t>v1.70.00 (T9b).</t>
+        </is>
+      </c>
+      <c r="G133" s="1" t="inlineStr">
+        <is>
+          <t>Gman request</t>
+        </is>
+      </c>
+      <c r="H133" s="3" t="n">
+        <v>46272</v>
+      </c>
+      <c r="I133" s="1" t="n"/>
+      <c r="J133" s="1" t="n"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="1" t="inlineStr">
+        <is>
+          <t>CM-166</t>
+        </is>
+      </c>
+      <c r="B134" s="1" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C134" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D134" s="1" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="E134" s="2" t="inlineStr">
+        <is>
+          <t>ROCm self-check cosmetic: 'failed to run offload-arch' warning</t>
+        </is>
+      </c>
+      <c r="F134" s="2" t="inlineStr">
+        <is>
+          <t>First line of every ROCm start. Suppress or explain.</t>
+        </is>
+      </c>
+      <c r="G134" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="H134" s="3" t="n">
+        <v>46272</v>
+      </c>
+      <c r="I134" s="1" t="n"/>
+      <c r="J134" s="1" t="n"/>
+    </row>
+    <row r="135" hidden="1" ht="30" customHeight="1">
+      <c r="A135" s="1" t="inlineStr">
+        <is>
+          <t>CM-167</t>
+        </is>
+      </c>
+      <c r="B135" s="1" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C135" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D135" s="1" t="inlineStr">
+        <is>
+          <t>Encode</t>
+        </is>
+      </c>
+      <c r="E135" s="2" t="inlineStr">
+        <is>
+          <t>AMF encoder probe frame too small (every AMD user encoded on the CPU)</t>
+        </is>
+      </c>
+      <c r="F135" s="2" t="inlineStr">
+        <is>
+          <t>Probe 640x360 nv12; failing probe prints its first stderr line. v1.70.00 (T8a). segB 27m44s -&gt; 10m25s.</t>
+        </is>
+      </c>
+      <c r="G135" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="H135" s="3" t="n">
+        <v>46272</v>
+      </c>
+      <c r="I135" s="1" t="n"/>
+      <c r="J135" s="1" t="n"/>
+    </row>
+    <row r="136" hidden="1">
+      <c r="A136" s="1" t="inlineStr">
+        <is>
+          <t>CM-168</t>
+        </is>
+      </c>
+      <c r="B136" s="1" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C136" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D136" s="1" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="E136" s="2" t="inlineStr">
+        <is>
+          <t>MIOpen cache pinned next to the exe</t>
+        </is>
+      </c>
+      <c r="F136" s="2" t="inlineStr">
+        <is>
+          <t>Survives updates; first-run compile notice. v1.70.00 (T9b).</t>
+        </is>
+      </c>
+      <c r="G136" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="H136" s="3" t="n">
+        <v>46272</v>
+      </c>
+      <c r="I136" s="1" t="n"/>
+      <c r="J136" s="1" t="n"/>
+    </row>
+    <row r="137" hidden="1" ht="30" customHeight="1">
+      <c r="A137" s="1" t="inlineStr">
+        <is>
+          <t>CM-169</t>
+        </is>
+      </c>
+      <c r="B137" s="1" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C137" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D137" s="1" t="inlineStr">
+        <is>
+          <t>Detection</t>
+        </is>
+      </c>
+      <c r="E137" s="2" t="inlineStr">
+        <is>
+          <t>ROCm forces Detection FP16 off</t>
+        </is>
+      </c>
+      <c r="F137" s="2" t="inlineStr">
+        <is>
+          <t>FP16 detection stops detecting after the first frames on the 9060 XT. Greyed with reason. v1.70.00 (T8a). Restoration FP16 was left live on a 270-frame test -&gt; CM-186.</t>
+        </is>
+      </c>
+      <c r="G137" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="H137" s="3" t="n">
+        <v>46272</v>
+      </c>
+      <c r="I137" s="1" t="n"/>
+      <c r="J137" s="1" t="n"/>
+    </row>
+    <row r="138" hidden="1">
+      <c r="A138" s="1" t="inlineStr">
+        <is>
+          <t>CM-170</t>
+        </is>
+      </c>
+      <c r="B138" s="1" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C138" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D138" s="1" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="E138" s="2" t="inlineStr">
+        <is>
+          <t>ultralytics settings sync=False</t>
+        </is>
+      </c>
+      <c r="F138" s="2" t="inlineStr">
+        <is>
+          <t>v1.70.00 (T9b).</t>
+        </is>
+      </c>
+      <c r="G138" s="1" t="inlineStr">
+        <is>
+          <t>Claude Analysis</t>
+        </is>
+      </c>
+      <c r="H138" s="3" t="n">
+        <v>46272</v>
+      </c>
+      <c r="I138" s="1" t="n"/>
+      <c r="J138" s="1" t="n"/>
+    </row>
+    <row r="139" ht="60" customHeight="1">
+      <c r="A139" s="1" t="inlineStr">
+        <is>
+          <t>CM-171</t>
+        </is>
+      </c>
+      <c r="B139" s="1" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C139" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D139" s="1" t="inlineStr">
+        <is>
+          <t>Decode</t>
+        </is>
+      </c>
+      <c r="E139" s="2" t="inlineStr">
+        <is>
+          <t>Decode transport: Windows anonymous pipe is the wall (AMD + Intel)</t>
+        </is>
+      </c>
+      <c r="F139" s="2" t="inlineStr">
+        <is>
+          <t>-probe-decode named it: decoder 447 fps, pipe 37-39 fps @1080p; 63% of the AMD wall, 60% of Intel. Fix: 64 MB pipe buffer (_winapi.CreatePipe) or named pipe; PyAV in-process as fallback rung. Expected AMD ~7h -&gt; ~5h50m, Intel -3.5h. rocDecode-for-Windows on STANDING WATCH. NEXT DROP.</t>
+        </is>
+      </c>
+      <c r="G139" s="1" t="inlineStr">
+        <is>
+          <t>Claude Analysis</t>
+        </is>
+      </c>
+      <c r="H139" s="3" t="n">
+        <v>46272</v>
+      </c>
+      <c r="I139" s="1" t="n"/>
+      <c r="J139" s="1" t="n"/>
+    </row>
+    <row r="140" hidden="1" ht="30" customHeight="1">
+      <c r="A140" s="1" t="inlineStr">
+        <is>
+          <t>CM-172</t>
+        </is>
+      </c>
+      <c r="B140" s="1" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C140" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D140" s="1" t="inlineStr">
+        <is>
+          <t>Mosaic</t>
+        </is>
+      </c>
+      <c r="E140" s="2" t="inlineStr">
+        <is>
+          <t>Per-shape MIOpen compiles in the blend mask (22-hour AMD collapse)</t>
+        </is>
+      </c>
+      <c r="F140" s="2" t="inlineStr">
+        <is>
+          <t>conv2d/avg_pool2d -&gt; summed-area box filter, verified to 2.5e-5 vs legacy. v1.70.00 (T9a). Intel: -21% restore on segB.</t>
+        </is>
+      </c>
+      <c r="G140" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="H140" s="3" t="n">
+        <v>46273</v>
+      </c>
+      <c r="I140" s="1" t="n"/>
+      <c r="J140" s="1" t="n"/>
+    </row>
+    <row r="141" hidden="1" ht="30" customHeight="1">
+      <c r="A141" s="1" t="inlineStr">
+        <is>
+          <t>CM-173</t>
+        </is>
+      </c>
+      <c r="B141" s="1" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C141" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D141" s="1" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="E141" s="2" t="inlineStr">
+        <is>
+          <t>Saved configurations (presets) in the gear menu</t>
+        </is>
+      </c>
+      <c r="F141" s="2" t="inlineStr">
+        <is>
+          <t>Whole-panel snapshots, one-click load, save-as/delete modal. v1.70.00 (T9e/T9f/T9g). Run-report 'panel' block reuses the schema (CM-180).</t>
+        </is>
+      </c>
+      <c r="G141" s="1" t="inlineStr">
+        <is>
+          <t>Gman request</t>
+        </is>
+      </c>
+      <c r="H141" s="3" t="n">
+        <v>46273</v>
+      </c>
+      <c r="I141" s="1" t="n"/>
+      <c r="J141" s="1" t="n"/>
+    </row>
+    <row r="142" ht="45" customHeight="1">
+      <c r="A142" s="1" t="inlineStr">
+        <is>
+          <t>CM-174</t>
+        </is>
+      </c>
+      <c r="B142" s="1" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C142" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D142" s="1" t="inlineStr">
+        <is>
+          <t>Encode</t>
+        </is>
+      </c>
+      <c r="E142" s="2" t="inlineStr">
+        <is>
+          <t>Remux watchdog vs +faststart in-place rewrite</t>
+        </is>
+      </c>
+      <c r="F142" s="2" t="inlineStr">
+        <is>
+          <t>No-growth kill on ~20 GB+ outputs during the faststart pass. Count mtime as progress + faststart allowance -- OR moot once CM-187 removes the pass. NEXT DROP (decide with CM-187).</t>
+        </is>
+      </c>
+      <c r="G142" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="H142" s="3" t="n">
+        <v>46274</v>
+      </c>
+      <c r="I142" s="1" t="n"/>
+      <c r="J142" s="1" t="n"/>
+    </row>
+    <row r="143" ht="45" customHeight="1">
+      <c r="A143" s="1" t="inlineStr">
+        <is>
+          <t>CM-175</t>
+        </is>
+      </c>
+      <c r="B143" s="1" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C143" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D143" s="1" t="inlineStr">
+        <is>
+          <t>Mosaic</t>
+        </is>
+      </c>
+      <c r="E143" s="2" t="inlineStr">
+        <is>
+          <t>4K VRAM reserve + Auto -&gt; host when the RAM plan fits</t>
+        </is>
+      </c>
+      <c r="F143" s="2" t="inlineStr">
+        <is>
+          <t>Reserve omits decoder 16-frame buffer (~400 MB @4K), NVENC surfaces (~300 MB), region transients; Auto picks host only when headroom &lt; 0. Folds into CM-155. NEXT DROP.</t>
+        </is>
+      </c>
+      <c r="G143" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="H143" s="3" t="n">
+        <v>46274</v>
+      </c>
+      <c r="I143" s="1" t="n"/>
+      <c r="J143" s="1" t="n"/>
+    </row>
+    <row r="144" ht="30" customHeight="1">
+      <c r="A144" s="1" t="inlineStr">
+        <is>
+          <t>CM-176</t>
+        </is>
+      </c>
+      <c r="B144" s="1" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C144" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D144" s="1" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="E144" s="2" t="inlineStr">
+        <is>
+          <t>faulthandler.enable() at the frozen entry</t>
+        </is>
+      </c>
+      <c r="F144" s="2" t="inlineStr">
+        <is>
+          <t>Native faults write the Python stack to the console log (drive-F: silent exit case). NEXT DROP.</t>
+        </is>
+      </c>
+      <c r="G144" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="H144" s="3" t="n">
+        <v>46274</v>
+      </c>
+      <c r="I144" s="1" t="n"/>
+      <c r="J144" s="1" t="n"/>
+    </row>
+    <row r="145" ht="30" customHeight="1">
+      <c r="A145" s="1" t="inlineStr">
+        <is>
+          <t>CM-177</t>
+        </is>
+      </c>
+      <c r="B145" s="1" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C145" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D145" s="1" t="inlineStr">
+        <is>
+          <t>Decode</t>
+        </is>
+      </c>
+      <c r="E145" s="2" t="inlineStr">
+        <is>
+          <t>Decoder frame-count sanity check per file</t>
+        </is>
+      </c>
+      <c r="F145" s="2" t="inlineStr">
+        <is>
+          <t>Demuxer count vs container duration wildly apart -&gt; stop the FILE with 'source unreadable -- check the drive', continue the batch. Absorbs CM-129. NEXT DROP.</t>
+        </is>
+      </c>
+      <c r="G145" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="H145" s="3" t="n">
+        <v>46274</v>
+      </c>
+      <c r="I145" s="1" t="n"/>
+      <c r="J145" s="1" t="n"/>
+    </row>
+    <row r="146" ht="45" customHeight="1">
+      <c r="A146" s="1" t="inlineStr">
+        <is>
+          <t>CM-178</t>
+        </is>
+      </c>
+      <c r="B146" s="1" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C146" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D146" s="1" t="inlineStr">
+        <is>
+          <t>Packaging</t>
+        </is>
+      </c>
+      <c r="E146" s="2" t="inlineStr">
+        <is>
+          <t>Per-edition build/dist folders</t>
+        </is>
+      </c>
+      <c r="F146" s="2" t="inlineStr">
+        <is>
+          <t>build-&lt;edition&gt;/dist-&lt;edition&gt; via spec workpath/distpath + the three .ps1; packager prints which tree it wrote. The NVIDIA patch zip existed only because NVIDIA was built last. NEXT DROP.</t>
+        </is>
+      </c>
+      <c r="G146" s="1" t="inlineStr">
+        <is>
+          <t>Gman request</t>
+        </is>
+      </c>
+      <c r="H146" s="3" t="n">
+        <v>46275</v>
+      </c>
+      <c r="I146" s="1" t="n"/>
+      <c r="J146" s="1" t="n"/>
+    </row>
+    <row r="147" ht="45" customHeight="1">
+      <c r="A147" s="1" t="inlineStr">
+        <is>
+          <t>CM-179</t>
+        </is>
+      </c>
+      <c r="B147" s="1" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C147" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D147" s="1" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="E147" s="2" t="inlineStr">
+        <is>
+          <t>Keep-awake held through finalize</t>
+        </is>
+      </c>
+      <c r="F147" s="2" t="inlineStr">
+        <is>
+          <t>pipeline.run releases the claim before EOF flush/remux -&gt; machine sleeps during long remux (mux=2316 s on two machines). Also hold ES_DISPLAY_REQUIRED (see CM-188). NEXT DROP.</t>
+        </is>
+      </c>
+      <c r="G147" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="H147" s="3" t="n">
+        <v>46275</v>
+      </c>
+      <c r="I147" s="1" t="n"/>
+      <c r="J147" s="1" t="n"/>
+    </row>
+    <row r="148" ht="90" customHeight="1">
+      <c r="A148" s="1" t="inlineStr">
+        <is>
+          <t>CM-180</t>
+        </is>
+      </c>
+      <c r="B148" s="1" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C148" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D148" s="1" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="E148" s="2" t="inlineStr">
+        <is>
+          <t>Run report replaces the misses JSON (spec written)</t>
+        </is>
+      </c>
+      <c r="F148" s="2" t="inlineStr">
+        <is>
+          <t>&lt;stem&gt;.run.json: 'panel' = the control panel exactly as submitted (preset schema; 'Load settings from a run...'), 'effective' = asked/ran/reason for every forced field, structured timing, counts, events, per-frame lists as ranges, whole console to &lt;stem&gt;.log; runReport = beside|temp|off. Absorbs CM-185. Spec: claude/ChitraMaya-CM180-RunReport-Spec.md. Three OPEN decisions for Gman. User request (forum) for the off switch. NEXT DROP.</t>
+        </is>
+      </c>
+      <c r="G148" s="1" t="inlineStr">
+        <is>
+          <t>Gman request</t>
+        </is>
+      </c>
+      <c r="H148" s="3" t="n">
+        <v>46275</v>
+      </c>
+      <c r="I148" s="1" t="n"/>
+      <c r="J148" s="1" t="n"/>
+    </row>
+    <row r="149" ht="45" customHeight="1">
+      <c r="A149" s="1" t="inlineStr">
+        <is>
+          <t>CM-181</t>
+        </is>
+      </c>
+      <c r="B149" s="1" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C149" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D149" s="1" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="E149" s="2" t="inlineStr">
+        <is>
+          <t>lada _full.pth = training checkpoint: label/skip + mmengine message</t>
+        </is>
+      </c>
+      <c r="F149" s="2" t="inlineStr">
+        <is>
+          <t>Manage Models lists all 17 lada files; 'download all, compile all' pulls the 287 MB training checkpoint (needs mmengine, never shipped). Label it, skip it in Compile All, loader message names mmengine. From GitHub issue #7's class of user. NEXT DROP.</t>
+        </is>
+      </c>
+      <c r="G149" s="1" t="inlineStr">
+        <is>
+          <t>GitHub issue #7</t>
+        </is>
+      </c>
+      <c r="H149" s="3" t="n">
+        <v>46275</v>
+      </c>
+      <c r="I149" s="1" t="n"/>
+      <c r="J149" s="1" t="inlineStr">
+        <is>
+          <t>https://github.com/seatv/ChitraMaya/issues/7</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="30" customHeight="1">
+      <c r="A150" s="1" t="inlineStr">
+        <is>
+          <t>CM-182</t>
+        </is>
+      </c>
+      <c r="B150" s="1" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C150" s="1" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="D150" s="1" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="E150" s="2" t="inlineStr">
+        <is>
+          <t>Multi-language UI</t>
+        </is>
+      </c>
+      <c r="F150" s="2" t="inlineStr">
+        <is>
+          <t>Strings table + data-i18n + language key; console stays English; ask which language; community translations via the hub. | 2026-09-14: FIRST TRANSLATIONS RECEIVED -- zh-CN and zh-TW (CSV + JSON), 342/342 keys, no empties, placeholders intact, 11 entries legitimately untranslated (FPS, FP16, HEVC, IoU, SBS, data.yaml, FB/FF); zh-TW is a real localization (64/342 identical to zh-CN), not a script conversion. Remaining work is ours: language switch + string loader in the UI (data-i18n on the extracted keys), fallback to English per key, RTL not needed yet. Gman moved to P1.</t>
+        </is>
+      </c>
+      <c r="G150" s="1" t="inlineStr">
+        <is>
+          <t>User request (forum)</t>
+        </is>
+      </c>
+      <c r="H150" s="3" t="n">
+        <v>46275</v>
+      </c>
+      <c r="I150" s="1" t="n"/>
+      <c r="J150" s="1" t="n"/>
+    </row>
+    <row r="151" ht="30" customHeight="1">
+      <c r="A151" s="1" t="inlineStr">
+        <is>
+          <t>CM-183</t>
+        </is>
+      </c>
+      <c r="B151" s="1" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C151" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D151" s="1" t="inlineStr">
+        <is>
+          <t>Detection</t>
+        </is>
+      </c>
+      <c r="E151" s="2" t="inlineStr">
+        <is>
+          <t>Compile defaults scaled to free VRAM</t>
+        </is>
+      </c>
+      <c r="F151" s="2" t="inlineStr">
+        <is>
+          <t>Fixed max-batch 8 / workspace 2 GB overflow 4 GB cards (TRT OOM tactic skips). Derive from free VRAM; expose in the compile modal. NEXT DROP.</t>
+        </is>
+      </c>
+      <c r="G151" s="1" t="inlineStr">
+        <is>
+          <t>GitHub issue #7</t>
+        </is>
+      </c>
+      <c r="H151" s="3" t="n">
+        <v>46275</v>
+      </c>
+      <c r="I151" s="1" t="n"/>
+      <c r="J151" s="1" t="inlineStr">
+        <is>
+          <t>https://github.com/seatv/ChitraMaya/issues/7</t>
+        </is>
+      </c>
+    </row>
+    <row r="152" ht="60" customHeight="1">
+      <c r="A152" s="1" t="inlineStr">
+        <is>
+          <t>CM-184</t>
+        </is>
+      </c>
+      <c r="B152" s="1" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C152" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D152" s="1" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="E152" s="2" t="inlineStr">
+        <is>
+          <t>Hide RTX Super-Res on AMD/Intel; RTX -&gt; ESRGAN fallback</t>
+        </is>
+      </c>
+      <c r="F152" s="2" t="inlineStr">
+        <is>
+          <t>rtx-2x/4x offered on every edition; on AMD the request fails and the run continues with NO secondary after one warning line; NVIDIA-saved configs carry it in. Remove on rocm/xpu, map to esrgan-4x with a console line, fall back to ESRGAN (not nothing) when the RTX runtime is missing. NEXT DROP.</t>
+        </is>
+      </c>
+      <c r="G152" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="H152" s="3" t="n">
+        <v>46275</v>
+      </c>
+      <c r="I152" s="1" t="n"/>
+      <c r="J152" s="1" t="n"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="1" t="inlineStr">
+        <is>
+          <t>CM-185</t>
+        </is>
+      </c>
+      <c r="B153" s="1" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C153" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D153" s="1" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="E153" s="2" t="inlineStr">
+        <is>
+          <t>Echo blend mask in the request line and the run report</t>
+        </is>
+      </c>
+      <c r="F153" s="2" t="inlineStr">
+        <is>
+          <t>Absorbed by CM-180.</t>
+        </is>
+      </c>
+      <c r="G153" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="H153" s="3" t="n">
+        <v>46275</v>
+      </c>
+      <c r="I153" s="1" t="n"/>
+      <c r="J153" s="1" t="n"/>
+    </row>
+    <row r="154" ht="75" customHeight="1">
+      <c r="A154" s="1" t="inlineStr">
+        <is>
+          <t>CM-186</t>
+        </is>
+      </c>
+      <c r="B154" s="1" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C154" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D154" s="1" t="inlineStr">
+        <is>
+          <t>Mosaic</t>
+        </is>
+      </c>
+      <c r="E154" s="2" t="inlineStr">
+        <is>
+          <t>Restoration FP16 fence on ROCm + non-finite/black output guard (all editions)</t>
+        </is>
+      </c>
+      <c r="F154" s="2" t="inlineStr">
+        <is>
+          <t>ROCm forces restoration FP16 off (greyed + reason, like CM-169); every edition checks each restored chunk for non-finite / all-zero before paste-back -&gt; redo in FP32 + warning + report event. Black-box cause NOT confirmed as FP16 (see CM-188); this is defence in depth. README/notes currently say Restoration FP16 'works and is your choice' and the toggle defaults on -&gt; correct with the drop. NEXT DROP.</t>
+        </is>
+      </c>
+      <c r="G154" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="H154" s="3" t="n">
+        <v>46276</v>
+      </c>
+      <c r="I154" s="1" t="n"/>
+      <c r="J154" s="1" t="n"/>
+    </row>
+    <row r="155" ht="105" customHeight="1">
+      <c r="A155" s="1" t="inlineStr">
+        <is>
+          <t>CM-187</t>
+        </is>
+      </c>
+      <c r="B155" s="1" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C155" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D155" s="1" t="inlineStr">
+        <is>
+          <t>Encode</t>
+        </is>
+      </c>
+      <c r="E155" s="2" t="inlineStr">
+        <is>
+          <t>One-pass finalize (audio extracted at run start; no vtmp; no faststart rewrite)</t>
+        </is>
+      </c>
+      <c r="F155" s="2" t="inlineStr">
+        <is>
+          <t>Finalize makes 9 whole-file passes on NVIDIA / 7 on AMD-Intel (~150 GB of disk traffic for a 31 GB 4K output) -&gt; watchdog kills -&gt; hand-fix every 4K remux. Extract audio once to &lt;stem&gt;.audio.mka (ride the ffmpeg decode pass on AMD/Intel); A/V offset via setts bsf on the stream-copied raw input (fallback -ss on audio); faststart via reserve_index_space (fallback none). 9-&gt;3 / 7-&gt;3 passes; CM-174 moot; RECOVER no longer needs the source. Verify per edition on segB (offset + no-offset) and one 4K on the Dell. Gman: discuss after the AMD investigation.</t>
+        </is>
+      </c>
+      <c r="G155" s="1" t="inlineStr">
+        <is>
+          <t>Gman + Claude</t>
+        </is>
+      </c>
+      <c r="H155" s="3" t="n">
+        <v>46276</v>
+      </c>
+      <c r="I155" s="1" t="n"/>
+      <c r="J155" s="1" t="n"/>
+    </row>
+    <row r="156" ht="90" customHeight="1">
+      <c r="A156" s="1" t="inlineStr">
+        <is>
+          <t>CM-188</t>
+        </is>
+      </c>
+      <c r="B156" s="1" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C156" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D156" s="1" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="E156" s="2" t="inlineStr">
+        <is>
+          <t>Detect GPU device reset / power event during a run; hold display-required</t>
+        </is>
+      </c>
+      <c r="F156" s="2" t="inlineStr">
+        <is>
+          <t>Black boxes + waviness appeared only in two UNATTENDED overnight AMD runs; no settings combination reproduces them (40-min, 45-min, full-title re-runs clean). Working theory: display-off / power-state / driver TDR (Event 4101 amdkmdag) / Windows Update mid-run -&gt; VRAM undefined, process survives. Check Event Viewer for the two windows. Fix: ES_DISPLAY_REQUIRED + system-required while running; detect device reset and abort loudly rather than continue with corrupted memory.</t>
+        </is>
+      </c>
+      <c r="G156" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="H156" s="3" t="n">
+        <v>46276</v>
+      </c>
+      <c r="I156" s="1" t="n"/>
+      <c r="J156" s="1" t="n"/>
+    </row>
+    <row r="157" ht="165" customHeight="1">
+      <c r="A157" s="1" t="inlineStr">
+        <is>
+          <t>CM-189</t>
+        </is>
+      </c>
+      <c r="B157" s="1" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C157" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D157" s="1" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="E157" s="2" t="inlineStr">
+        <is>
+          <t>Linux port (clone + pip + python -m chitramaya)</t>
+        </is>
+      </c>
+      <c r="F157" s="2" t="inlineStr">
+        <is>
+          <t>Code is largely OS-neutral (pathlib; engine suffix .win/.linux already exists). Windows couplings confined to winproc.py, keep_awake.py, gpu_gate.py (MessageBoxW + WMI), self_check.py (powershell GPU inventory), rtx_secondary.py (guarded). Gaps: pywebview needs GTK/Qt or a browser-only mode; hwaccel ladder lacks cuda/vaapi (lands on CPU decode); Maxine unavailable (optional). Plan: (1) sandbox smoke test with CPU torch -- import surface, -self-check, browser-mode UI, jsdom -- next release cycle; (2) driver-install walkthrough with Gman on the dual-boot box (Ubuntu 24.04 LTS; 9060 XT stays in the 3600XT box on PCIe 4.0 x16; 5600 + 32 GB coming from Seattle); (3) guards + hwaccel + docs/linux.md; (4) Linux release at some point, no date. Note: 63 unique cloners/14 days, spiking on push days = mostly automated cloners; some are people.</t>
+        </is>
+      </c>
+      <c r="G157" s="1" t="inlineStr">
+        <is>
+          <t>Gman + Claude</t>
+        </is>
+      </c>
+      <c r="H157" s="3" t="n">
+        <v>46276</v>
+      </c>
+      <c r="I157" s="1" t="n"/>
+      <c r="J157" s="1" t="n"/>
+    </row>
+    <row r="158" hidden="1" ht="45" customHeight="1">
+      <c r="A158" s="1" t="inlineStr">
+        <is>
+          <t>CM-190</t>
+        </is>
+      </c>
+      <c r="B158" s="1" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C158" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D158" s="1" t="inlineStr">
+        <is>
+          <t>Decode</t>
+        </is>
+      </c>
+      <c r="E158" s="2" t="inlineStr">
+        <is>
+          <t>MPEG-TS temp remux failed silently since v1.61 (.part suffix hid .mp4 from ffmpeg)</t>
+        </is>
+      </c>
+      <c r="F158" s="2" t="inlineStr">
+        <is>
+          <t>The CM-125 .part suffix made ffmpeg 'unable to choose an output format' for the CM-120 CFR temp, so every TS source was NVDEC-decoded directly with drops (head skip + gap-fill duplicates). Fixed 09-12 (T10a-2); remux temp in Temp; one console line names it.</t>
+        </is>
+      </c>
+      <c r="G158" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="H158" s="3" t="n">
+        <v>46277</v>
+      </c>
+    </row>
+    <row r="159" hidden="1" ht="135" customHeight="1">
+      <c r="A159" s="1" t="inlineStr">
+        <is>
+          <t>CM-191</t>
+        </is>
+      </c>
+      <c r="B159" s="1" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C159" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D159" s="1" t="inlineStr">
+        <is>
+          <t>Mosaic</t>
+        </is>
+      </c>
+      <c r="E159" s="2" t="inlineStr">
+        <is>
+          <t>Re-decode frame source (no frame store): second NVDEC decoder re-produces frames at paste-back time</t>
+        </is>
+      </c>
+      <c r="F159" s="2" t="inlineStr">
+        <is>
+          <t>Frames are not stored; the primary decoder feeds detection and cropping, a lagging Decoder on the same source (same backend/args; owns the TS remux temp) re-produces each frame when it is due for blend+encode. Alignment by frame number with PTS check (skip/freeze/count-only, counted). store_backend auto|redecode|device|host; auto -&gt; redecode on NVDEC (not VR projection / Test Frame). Field: byte-identical output vs the device store on PurpleRain, segB and a 4-min dense 4K cut; 2.8x faster than the device store on 8 GB; VRAM 11.06 -&gt; 7.86 GB on the 12 GB box. Design note: claude/ChitraMaya-CM191-RedecodeDesign.md. Shipped T10c/T10d/T10d-2.</t>
+        </is>
+      </c>
+      <c r="G159" s="1" t="inlineStr">
+        <is>
+          <t>Gman + Claude</t>
+        </is>
+      </c>
+      <c r="H159" s="3" t="n">
+        <v>46277</v>
+      </c>
+    </row>
+    <row r="160" ht="60" customHeight="1">
+      <c r="A160" s="1" t="inlineStr">
+        <is>
+          <t>CM-192</t>
+        </is>
+      </c>
+      <c r="B160" s="1" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C160" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D160" s="1" t="inlineStr">
+        <is>
+          <t>Mosaic</t>
+        </is>
+      </c>
+      <c r="E160" s="2" t="inlineStr">
+        <is>
+          <t>Auto clip window (goodbye MCL): cut clips at natural boundaries under a measured VRAM/quality ceiling</t>
+        </is>
+      </c>
+      <c r="F160" s="2" t="inlineStr">
+        <is>
+          <t>With frames free (CM-191) Max Clip Length no longer costs memory; cut clips at track end / TTL / shot change under an internal ceiling from the restorer's measured per-frame VRAM cost and a quality ceiling measured with ab_eval_noref at 60/120/180/300/600 on segB. Splash candidate; after CM-191 is proven on the Dell.</t>
+        </is>
+      </c>
+      <c r="G160" s="1" t="inlineStr">
+        <is>
+          <t>Gman + Claude</t>
+        </is>
+      </c>
+      <c r="H160" s="3" t="n">
+        <v>46277</v>
+      </c>
+    </row>
+    <row r="161" hidden="1" ht="75" customHeight="1">
+      <c r="A161" s="1" t="inlineStr">
+        <is>
+          <t>CM-193</t>
+        </is>
+      </c>
+      <c r="B161" s="1" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C161" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D161" s="1" t="inlineStr">
+        <is>
+          <t>Mosaic</t>
+        </is>
+      </c>
+      <c r="E161" s="2" t="inlineStr">
+        <is>
+          <t>Pending patches at clip resolution (unpad+resize at blend time)</t>
+        </is>
+      </c>
+      <c r="F161" s="2" t="inlineStr">
+        <is>
+          <t>Redecode patches were held at FRAME resolution: one 180-frame clip of 2400-px regions = 3.1 GB -&gt; the x16 8 GB run died at 59 % (CM-122). Patches now keep the restorer output at clip resolution (post-secondary, pre-unpad/resize); unpad+resize+blend run together at drain, same ops same order -&gt; bit-identical. ~570 MB per 180-frame clip with RTX 4x, ~47 MB without. Shipped T10d.</t>
+        </is>
+      </c>
+      <c r="G161" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="H161" s="3" t="n">
+        <v>46278</v>
+      </c>
+    </row>
+    <row r="162" hidden="1" ht="30" customHeight="1">
+      <c r="A162" s="1" t="inlineStr">
+        <is>
+          <t>CM-194</t>
+        </is>
+      </c>
+      <c r="B162" s="1" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C162" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D162" s="1" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="E162" s="2" t="inlineStr">
+        <is>
+          <t>Console drawer duplicated the startup block (overlapping polls)</t>
+        </is>
+      </c>
+      <c r="F162" s="2" t="inlineStr">
+        <is>
+          <t>One /api/console poll in flight at a time; an answer for a cursor already moved past is dropped. Shipped T10d.</t>
+        </is>
+      </c>
+      <c r="G162" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="H162" s="3" t="n">
+        <v>46278</v>
+      </c>
+    </row>
+    <row r="163" hidden="1" ht="60" customHeight="1">
+      <c r="A163" s="1" t="inlineStr">
+        <is>
+          <t>CM-195</t>
+        </is>
+      </c>
+      <c r="B163" s="1" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C163" s="1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D163" s="1" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="E163" s="2" t="inlineStr">
+        <is>
+          <t>Timestamped process console log, newest 20 kept</t>
+        </is>
+      </c>
+      <c r="F163" s="2" t="inlineStr">
+        <is>
+          <t>ChitraMaya-console-YYYYMMDD-HHMMSS[-pid].log in the app folder; older than the newest 20 deleted at launch; first console line names the file. Companion: CM-180 run report (&lt;stem&gt;.run.json + &lt;stem&gt;.log per run; runReport beside|temp|off). Shipped T10d.</t>
+        </is>
+      </c>
+      <c r="G163" s="1" t="inlineStr">
+        <is>
+          <t>Gman</t>
+        </is>
+      </c>
+      <c r="H163" s="3" t="n">
+        <v>46278</v>
+      </c>
+    </row>
+    <row r="164" hidden="1" ht="165" customHeight="1">
+      <c r="A164" s="1" t="inlineStr">
+        <is>
+          <t>CM-196</t>
+        </is>
+      </c>
+      <c r="B164" s="1" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C164" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="D164" s="1" t="inlineStr">
+        <is>
+          <t>Mosaic</t>
+        </is>
+      </c>
+      <c r="E164" s="2" t="inlineStr">
+        <is>
+          <t>8 GB VRAM oversubscription with the full stack: patches to pinned RAM, prefetch trims, VRAM ledger</t>
+        </is>
+      </c>
+      <c r="F164" s="2" t="inlineStr">
+        <is>
+          <t>Three NVENC error-8 deaths of one 4K60 title on 8 GB cards at its 2400-px regions; monitor: VRAM pinned at 7.9 GB from the first hour, WDDM paging 4 GB/s over OCuLink, 1.5-2 fps for 23 min before the lock failed. Fix (T10e, 3f68fee): pending patches wait in pinned host RAM (redecodePatches host|device, default host; byte copies, bit-exact); lag prefetch 8 -&gt; 4 frames; primary NVDEC prefetch 2x batch (min 8) on cards &lt; 10 GB; [VRAM] ledger lines (after models / first drain / end) with other = used - torch_reserved, vram column on every 500-frame checkpoint and in the run report; torch cache released after drains (rate-limited); run_error carries the exception text; effective.det_imgsz / redecode_patches. Field gate: segB device vs redecode on the Dell, then the full title with the monitor. If it still dies: the ledger names the next lever (denoise ultra / SS 4x footprint).</t>
+        </is>
+      </c>
+      <c r="G164" s="1" t="inlineStr">
+        <is>
+          <t>Field testing</t>
+        </is>
+      </c>
+      <c r="H164" s="3" t="n">
+        <v>46279</v>
+      </c>
+    </row>
+    <row r="165" ht="195" customHeight="1">
+      <c r="A165" s="1" t="inlineStr">
+        <is>
+          <t>CM-197</t>
+        </is>
+      </c>
+      <c r="B165" s="1" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C165" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D165" s="1" t="inlineStr">
+        <is>
+          <t>Mosaic</t>
+        </is>
+      </c>
+      <c r="E165" s="2" t="inlineStr">
+        <is>
+          <t>Two-pass restoration with a resumable plan (detect once, restore many; resume a dead run)</t>
+        </is>
+      </c>
+      <c r="F165" s="2" t="inlineStr">
+        <is>
+          <t>Pass 1: decode + detect + track only -&gt; a PLAN file: frame numbers, boxes, clip boundaries, masks (RLE/PNG or polygons; geometry only, no content, SFW by construction). Pass 2: decode + crop from the plan + restore + blend (lag decoder) + encode. Unlocks: RESUME a run that died mid-title from the plan at the last encoded frame (no other tool does this); detect once / restore N times with identical boxes for A/B; clip boundaries chosen with the whole timeline known (feeds CM-192); exact ETA from frame one; plan reusable by the CM-154 detector exam. Cost: one more NVDEC pass of the title (3 decodes instead of 2; the background engine, largely hidden) + plan I/O; detection is NOT repeated -- net wall time about even, possibly better from unbroken batches. Design questions: mask payload format; plan invalidation (source hash, detector model/imgsz/conf); resume = re-encode from plan + concatenate or continue the raw bitstream; UI: 'Resume' on a dead run's report. Gman 09-14: 'resume will be a great feature to have' -- schedule after prioritization, after T10e is proven.</t>
+        </is>
+      </c>
+      <c r="G165" s="1" t="inlineStr">
+        <is>
+          <t>Gman + Claude</t>
+        </is>
+      </c>
+      <c r="H165" s="3" t="n">
+        <v>46279</v>
+      </c>
+    </row>
+    <row r="166" ht="180" customHeight="1">
+      <c r="A166" s="1" t="inlineStr">
+        <is>
+          <t>CM-198</t>
+        </is>
+      </c>
+      <c r="B166" s="1" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C166" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D166" s="1" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="E166" s="2" t="inlineStr">
+        <is>
+          <t>nvGPUMonitor run trigger: monitor starts/stops with the run, CSV lands beside the run report</t>
+        </is>
+      </c>
+      <c r="F166" s="2" t="inlineStr">
+        <is>
+          <t>Today the monitor is started by hand and its CSV spans more than the run, so every analysis begins by slicing the window (the 09-14 Dell forensics) and half-runs get half a CSV (SegB-256 started midway). Integrate: the pipeline starts nvGPUMonitor at run start (a 'monitor' marker row) and stops it at finalize, CSV written as &lt;stem&gt;.monitor.csv beside &lt;stem&gt;.run.json; config key runMonitor on|off (default off until the exe ships with the app or its path is configured; monitorPath); the run report records monitor file + PCIe link (max_gen x cur_width) so the dial is right by construction. Also folds in the 09-14 monitor fixes: PCIe dial denominator = max_gen x cur_width (was max_gen x max_width: 15.76 GB/s shown for a Gen3 x4 link); per-sample NVML tx/rx peaks exceed the link maximum -&gt; smooth or label; decoder/encoder util read 0 on OCuLink eGPUs -&gt; mark n/a rather than 0. Gman 09-14: 'do we have a roadmap item to integrate nvGPUMonitor trigger?' -- no, this is it.</t>
+        </is>
+      </c>
+      <c r="G166" s="1" t="inlineStr">
+        <is>
+          <t>Gman + Claude</t>
+        </is>
+      </c>
+      <c r="H166" s="3" t="n">
+        <v>46279</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="1" t="inlineStr">
+        <is>
+          <t>CM-199</t>
+        </is>
+      </c>
+      <c r="B167" s="1" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C167" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D167" s="1" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="E167" s="2" t="inlineStr">
+        <is>
+          <t>Model hub: selectable Hugging Face endpoint (hf-mirror.com for China mainland) + automatic fallback</t>
+        </is>
+      </c>
+      <c r="F167" s="2" t="inlineStr">
+        <is>
+          <t>GitHub issue #13: huggingface.co needs a VPN from mainland China and is slow; hf-mirror.com is a free, fast reverse proxy with identical paths (/api/models/&lt;owner&gt;/&lt;repo&gt;/tree/main, /resolve/main/&lt;file&gt;). Our downloader hard-codes https://huggingface.co in three places (server.py: tree listing, resolve URL, token rule). Change: one endpoint value -- config key hfEndpoint in ChitraMaya-config.json (default https://huggingface.co), a dropdown in the model hub dialog (huggingface.co | hf-mirror.com (China mainland) | custom URL); model-sources.json keeps canonical huggingface.co URLs and the host is swapped at fetch time; the hf-token is sent only to the configured endpoint host; console line names the endpoint per download. Auto-fallback: a connection failure/timeout on huggingface.co retries once on hf-mirror.com and says so. Honouring HF_ENDPOINT as a default source is optional (Gman decides; env-var doctrine). README sentence in the Models section + zh-CN/zh-TW strings for the new dropdown (CM-182). Half a day; verify_ui_js/ui_smoke gates (dialog change).</t>
+        </is>
+      </c>
+      <c r="G167" s="1" t="inlineStr">
+        <is>
+          <t>GitHub #13</t>
+        </is>
+      </c>
+      <c r="H167" s="3" t="n">
+        <v>46279</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J91">
+  <autoFilter ref="A1:J166">
     <filterColumn colId="2" hiddenButton="0" showButton="1">
       <filters>
         <filter val="Open"/>
@@ -4284,4 +7478,609 @@
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Order</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Why now</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Size</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Needs from Gman</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>CM-179</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Keep-awake through finalize</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Two machines slept during the remux; trivial change</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>hours</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>CM-187</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>One-pass finalize</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Every 4K remux hand-fixed; removes CM-174's failure mode</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1-2 days</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>OPEN: discuss after AMD; approve the design</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>CM-186</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Restoration FP16 fence + black-output guard</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Defence in depth; docs say the opposite today</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>half day</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Confirm ESRGAN-on run looks right</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>CM-184</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Hide RTX on AMD/Intel, ESRGAN fallback</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Silent no-secondary runs from imported configs</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>hours</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>CM-180</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Run report (panel + effective)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Could not tell what ran; user asked for the off switch</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>1-2 days</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>3 OPEN decisions in the spec</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>CM-171</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Pipe transport</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>63% of the AMD wall, 60% of Intel</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>1 day + measurement</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>AMD box available for segB before teardown?</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>CM-175 / CM-155</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>VRAM reserve + Auto-&gt;host / planner clamp</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Dell 8GB@4K died twice on the device store</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>1 day</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>CM-151 + CM-183</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Engine manifest, warnings badge, compile defaults from VRAM</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>GitHub issue #7 open on it</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>1-2 days</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CM-181</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>_full checkpoint label/skip + mmengine message</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Same user class as #7</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>hours</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>CM-176 / CM-177</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>faulthandler + decoder frame-count sanity</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Drive-F: silent exit</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>half day</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>CM-178</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Per-edition build/dist</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Release-day lesson</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>hours</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>hwDecode key</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Config key -&gt; CM_HW_DECODE</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Env-var doctrine; README documented a key that never existed</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>hour</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>CM-086</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Facefusion blend: fix or drop</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Confirmed noise source 09-11</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>half day</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Decide fix vs drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>misc</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>CM-166; probe prints cuda on ROCm; errored-run decoder warning</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>nits</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>hours</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>CM-188</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Device-reset detection + display-required</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Depends on the Event Viewer finding</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>half day</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Event Viewer check for the two overnight windows</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="160" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Roadmap brought forward from CM-090 (2026-07-28) to CM-188 (2026-09-11).</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Existing rows updated: CM-046/061/074/084/087/088/090 -&gt; Done; CM-047 -&gt; superseded by CM-151; CM-062 -&gt; largely superseded; CM-086 -&gt; P1, confirmed 09-11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CM IDs known to be parked but whose titles were not recovered in this pass: CM-092, 094, 096-102, 106-108, 110-111, 113, 115-118, 121-123, 133-135, 137-138, 140, 143-145, 147. Fill from the batch notes or drop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Status values used: Done / Open / In progress. Priorities are PROPOSED for new rows; Gman decides.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>'Next Drop (proposed)' is an ordering for review, not a commitment. Items marked NEXT DROP in the Description column match it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Release rule (09-11): no release without watching and approving a full studio-mosaic restoration on each edition released.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Phase C rule (09-11): no model leaves the lab on numbers alone -- watch a full studio-mosaic restoration vs generic first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-09-14: rows CM-190..CM-197 added (post-release drops T10a..T10e). Statuses: 190/191/193/194/195 Done in the field; 196 Field testing (T10e built, Dell gate pending); 192 Open; 197 NEW -- two-pass plan + resume, added at Gman's request 09-14, to be prioritized.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-14: CM-186 shipped as the black-output guard only (no FP16 fence -- no proof FP16 hurts restoration on AMD); CM-187 + CM-179 shipped in T10a (one-pass finalize). Mark Done when the release goes out.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-14 PM: CM-198 added (nvGPUMonitor run trigger + the PCIe dial fix). 256/512 study on segB: 512 = poor reconstruction with the generic v1.2 weights -&gt; a larger clip needs its own trained weights (Phase C); recorded in the day state.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-14 PM (merge): Gman's priority changes kept (CM-038 P1, CM-182 P1; CM-083/086/186/188 -&gt; P2); CM-182 -&gt; In progress with the zh-CN/zh-TW delivery noted. CM-198 was already in Gman's copy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-14 PM: CM-199 added from GitHub issue #13 (hf-mirror.com endpoint for the model hub).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>